<commit_message>
formatter for excel improved
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -427,10 +427,6 @@
   </sheetPr>
   <dimension ref="A1:A101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">

</xml_diff>